<commit_message>
Elabora Resumo e Resultados do iGovTI 2026, insere referencias a graficos por esfera e adiciona scripts de automacao e validacao
</commit_message>
<xml_diff>
--- a/02-Execucao/03-Execucao_Procedimentos/tabelas_consolidadas_auditoria.xlsx
+++ b/02-Execucao/03-Execucao_Procedimentos/tabelas_consolidadas_auditoria.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5776" uniqueCount="176">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5792" uniqueCount="176">
   <si>
     <t>1. Estrutura de TIC insuficiente para coordenar, gerir e sustentar a tecnologia da informação.</t>
   </si>
@@ -412,7 +412,7 @@
     <t>[Recomendação] designe formalmente equipe responsável pelo planejamento das contratações de TIC, atentando-se, minimamente, em assegurar a participação da área requisitante, da área técnica de TIC e das demais áreas necessárias, com definição das responsabilidades de seus integrantes</t>
   </si>
   <si>
-    <t>[Recomendação] estabeleça a submissão das contratações de TIC à análise prévia e à aprovação técnica da área de TIC, inclusive quando demandadas por outras áreas, de modo a verificar a compatibilidade da solução com os padrões tecnológicos, os requisitos institucionais, a segurança da informação e a arquitetura existente</t>
+    <t>[Recomendação] estabeleça a submissão das contratações de TIC à análise prévia e à aprovação técnica da área de TIC, inclusive quando demandadas por outras áreas, de modo a verificar a compatibilidade da solução com os padrões tecnológicos, os requisitos institucionais, a segurança da informação e a arquitetura existente, facultando a adoção de fluxos simplificados ou a dispensa de parecer detalhado para contratações diretas por dispensa em razão do valor (baixo valor) ou de baixa complexidade técnica, mediante critérios objetivos ou catálogos de soluções padronizadas</t>
   </si>
   <si>
     <t>[Recomendação] estabeleça e execute rotina periódica de acompanhamento, revisão e atualização do plano de TIC, atentando-se, minimamente, em registrar a execução das iniciativas, as pendências, as reprogramações e as deliberações adotadas</t>
@@ -3899,6 +3899,9 @@
       <c r="C8" t="s">
         <v>121</v>
       </c>
+      <c r="D8" t="s">
+        <v>121</v>
+      </c>
       <c r="E8" t="s">
         <v>121</v>
       </c>
@@ -3914,6 +3917,12 @@
       <c r="I8" t="s">
         <v>121</v>
       </c>
+      <c r="J8" t="s">
+        <v>121</v>
+      </c>
+      <c r="K8" t="s">
+        <v>121</v>
+      </c>
       <c r="L8" t="s">
         <v>121</v>
       </c>
@@ -3924,6 +3933,9 @@
         <v>121</v>
       </c>
       <c r="O8" t="s">
+        <v>121</v>
+      </c>
+      <c r="P8" t="s">
         <v>121</v>
       </c>
       <c r="Q8" t="s">
@@ -4669,6 +4681,9 @@
       <c r="C21" t="s">
         <v>121</v>
       </c>
+      <c r="D21" t="s">
+        <v>121</v>
+      </c>
       <c r="E21" t="s">
         <v>121</v>
       </c>
@@ -4684,6 +4699,12 @@
       <c r="I21" t="s">
         <v>121</v>
       </c>
+      <c r="J21" t="s">
+        <v>121</v>
+      </c>
+      <c r="K21" t="s">
+        <v>121</v>
+      </c>
       <c r="L21" t="s">
         <v>121</v>
       </c>
@@ -4694,6 +4715,9 @@
         <v>121</v>
       </c>
       <c r="O21" t="s">
+        <v>121</v>
+      </c>
+      <c r="P21" t="s">
         <v>121</v>
       </c>
       <c r="Q21" t="s">
@@ -11498,6 +11522,9 @@
       <c r="A8" s="1" t="s">
         <v>13</v>
       </c>
+      <c r="B8" t="s">
+        <v>121</v>
+      </c>
       <c r="C8" t="s">
         <v>121</v>
       </c>
@@ -11534,6 +11561,9 @@
       <c r="N8" t="s">
         <v>121</v>
       </c>
+      <c r="O8" t="s">
+        <v>121</v>
+      </c>
       <c r="P8" t="s">
         <v>121</v>
       </c>
@@ -11561,7 +11591,13 @@
       <c r="X8" t="s">
         <v>121</v>
       </c>
+      <c r="Y8" t="s">
+        <v>121</v>
+      </c>
       <c r="Z8" t="s">
+        <v>121</v>
+      </c>
+      <c r="AA8" t="s">
         <v>121</v>
       </c>
     </row>
@@ -12268,6 +12304,9 @@
       <c r="A21" s="1" t="s">
         <v>26</v>
       </c>
+      <c r="B21" t="s">
+        <v>121</v>
+      </c>
       <c r="C21" t="s">
         <v>121</v>
       </c>
@@ -12304,6 +12343,9 @@
       <c r="N21" t="s">
         <v>121</v>
       </c>
+      <c r="O21" t="s">
+        <v>121</v>
+      </c>
       <c r="P21" t="s">
         <v>121</v>
       </c>
@@ -12331,7 +12373,13 @@
       <c r="X21" t="s">
         <v>121</v>
       </c>
+      <c r="Y21" t="s">
+        <v>121</v>
+      </c>
       <c r="Z21" t="s">
+        <v>121</v>
+      </c>
+      <c r="AA21" t="s">
         <v>121</v>
       </c>
     </row>
@@ -18615,7 +18663,7 @@
     </row>
     <row r="2" spans="1:3">
       <c r="A2" s="1" t="s">
-        <v>35</v>
+        <v>13</v>
       </c>
       <c r="B2">
         <v>6</v>
@@ -18626,7 +18674,7 @@
     </row>
     <row r="3" spans="1:3">
       <c r="A3" s="1" t="s">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="B3">
         <v>6</v>
@@ -18637,7 +18685,7 @@
     </row>
     <row r="4" spans="1:3">
       <c r="A4" s="1" t="s">
-        <v>84</v>
+        <v>35</v>
       </c>
       <c r="B4">
         <v>6</v>
@@ -18648,7 +18696,7 @@
     </row>
     <row r="5" spans="1:3">
       <c r="A5" s="1" t="s">
-        <v>114</v>
+        <v>38</v>
       </c>
       <c r="B5">
         <v>6</v>
@@ -18659,29 +18707,29 @@
     </row>
     <row r="6" spans="1:3">
       <c r="A6" s="1" t="s">
-        <v>10</v>
+        <v>84</v>
       </c>
       <c r="B6">
         <v>6</v>
       </c>
       <c r="C6">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" s="1" t="s">
-        <v>11</v>
+        <v>114</v>
       </c>
       <c r="B7">
         <v>6</v>
       </c>
       <c r="C7">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" s="1" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="B8">
         <v>6</v>
@@ -18692,7 +18740,7 @@
     </row>
     <row r="9" spans="1:3">
       <c r="A9" s="1" t="s">
-        <v>60</v>
+        <v>11</v>
       </c>
       <c r="B9">
         <v>6</v>
@@ -18703,7 +18751,7 @@
     </row>
     <row r="10" spans="1:3">
       <c r="A10" s="1" t="s">
-        <v>87</v>
+        <v>14</v>
       </c>
       <c r="B10">
         <v>6</v>
@@ -18714,7 +18762,7 @@
     </row>
     <row r="11" spans="1:3">
       <c r="A11" s="1" t="s">
-        <v>88</v>
+        <v>60</v>
       </c>
       <c r="B11">
         <v>6</v>
@@ -18725,7 +18773,7 @@
     </row>
     <row r="12" spans="1:3">
       <c r="A12" s="1" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B12">
         <v>6</v>
@@ -18736,7 +18784,7 @@
     </row>
     <row r="13" spans="1:3">
       <c r="A13" s="1" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="B13">
         <v>6</v>
@@ -18747,7 +18795,7 @@
     </row>
     <row r="14" spans="1:3">
       <c r="A14" s="1" t="s">
-        <v>98</v>
+        <v>89</v>
       </c>
       <c r="B14">
         <v>6</v>
@@ -18758,7 +18806,7 @@
     </row>
     <row r="15" spans="1:3">
       <c r="A15" s="1" t="s">
-        <v>100</v>
+        <v>93</v>
       </c>
       <c r="B15">
         <v>6</v>
@@ -18769,7 +18817,7 @@
     </row>
     <row r="16" spans="1:3">
       <c r="A16" s="1" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="B16">
         <v>6</v>
@@ -18780,7 +18828,7 @@
     </row>
     <row r="17" spans="1:3">
       <c r="A17" s="1" t="s">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="B17">
         <v>6</v>
@@ -18791,7 +18839,7 @@
     </row>
     <row r="18" spans="1:3">
       <c r="A18" s="1" t="s">
-        <v>115</v>
+        <v>104</v>
       </c>
       <c r="B18">
         <v>6</v>
@@ -18802,7 +18850,7 @@
     </row>
     <row r="19" spans="1:3">
       <c r="A19" s="1" t="s">
-        <v>117</v>
+        <v>108</v>
       </c>
       <c r="B19">
         <v>6</v>
@@ -18813,7 +18861,7 @@
     </row>
     <row r="20" spans="1:3">
       <c r="A20" s="1" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="B20">
         <v>6</v>
@@ -18824,29 +18872,29 @@
     </row>
     <row r="21" spans="1:3">
       <c r="A21" s="1" t="s">
-        <v>20</v>
+        <v>117</v>
       </c>
       <c r="B21">
         <v>6</v>
       </c>
       <c r="C21">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="22" spans="1:3">
       <c r="A22" s="1" t="s">
-        <v>29</v>
+        <v>118</v>
       </c>
       <c r="B22">
         <v>6</v>
       </c>
       <c r="C22">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="23" spans="1:3">
       <c r="A23" s="1" t="s">
-        <v>56</v>
+        <v>20</v>
       </c>
       <c r="B23">
         <v>6</v>
@@ -18857,7 +18905,7 @@
     </row>
     <row r="24" spans="1:3">
       <c r="A24" s="1" t="s">
-        <v>92</v>
+        <v>29</v>
       </c>
       <c r="B24">
         <v>6</v>
@@ -18868,7 +18916,7 @@
     </row>
     <row r="25" spans="1:3">
       <c r="A25" s="1" t="s">
-        <v>106</v>
+        <v>56</v>
       </c>
       <c r="B25">
         <v>6</v>
@@ -18879,7 +18927,7 @@
     </row>
     <row r="26" spans="1:3">
       <c r="A26" s="1" t="s">
-        <v>107</v>
+        <v>92</v>
       </c>
       <c r="B26">
         <v>6</v>
@@ -18890,7 +18938,7 @@
     </row>
     <row r="27" spans="1:3">
       <c r="A27" s="1" t="s">
-        <v>113</v>
+        <v>106</v>
       </c>
       <c r="B27">
         <v>6</v>
@@ -18901,29 +18949,29 @@
     </row>
     <row r="28" spans="1:3">
       <c r="A28" s="1" t="s">
-        <v>9</v>
+        <v>107</v>
       </c>
       <c r="B28">
         <v>6</v>
       </c>
       <c r="C28">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="29" spans="1:3">
       <c r="A29" s="1" t="s">
-        <v>31</v>
+        <v>113</v>
       </c>
       <c r="B29">
         <v>6</v>
       </c>
       <c r="C29">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="30" spans="1:3">
       <c r="A30" s="1" t="s">
-        <v>51</v>
+        <v>9</v>
       </c>
       <c r="B30">
         <v>6</v>
@@ -18934,7 +18982,7 @@
     </row>
     <row r="31" spans="1:3">
       <c r="A31" s="1" t="s">
-        <v>63</v>
+        <v>31</v>
       </c>
       <c r="B31">
         <v>6</v>
@@ -18945,7 +18993,7 @@
     </row>
     <row r="32" spans="1:3">
       <c r="A32" s="1" t="s">
-        <v>66</v>
+        <v>51</v>
       </c>
       <c r="B32">
         <v>6</v>
@@ -18956,7 +19004,7 @@
     </row>
     <row r="33" spans="1:3">
       <c r="A33" s="1" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="B33">
         <v>6</v>
@@ -18967,7 +19015,7 @@
     </row>
     <row r="34" spans="1:3">
       <c r="A34" s="1" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="B34">
         <v>6</v>
@@ -18978,7 +19026,7 @@
     </row>
     <row r="35" spans="1:3">
       <c r="A35" s="1" t="s">
-        <v>81</v>
+        <v>70</v>
       </c>
       <c r="B35">
         <v>6</v>
@@ -18989,7 +19037,7 @@
     </row>
     <row r="36" spans="1:3">
       <c r="A36" s="1" t="s">
-        <v>90</v>
+        <v>71</v>
       </c>
       <c r="B36">
         <v>6</v>
@@ -19000,7 +19048,7 @@
     </row>
     <row r="37" spans="1:3">
       <c r="A37" s="1" t="s">
-        <v>96</v>
+        <v>81</v>
       </c>
       <c r="B37">
         <v>6</v>
@@ -19011,7 +19059,7 @@
     </row>
     <row r="38" spans="1:3">
       <c r="A38" s="1" t="s">
-        <v>109</v>
+        <v>90</v>
       </c>
       <c r="B38">
         <v>6</v>
@@ -19022,7 +19070,7 @@
     </row>
     <row r="39" spans="1:3">
       <c r="A39" s="1" t="s">
-        <v>120</v>
+        <v>96</v>
       </c>
       <c r="B39">
         <v>6</v>
@@ -19033,24 +19081,24 @@
     </row>
     <row r="40" spans="1:3">
       <c r="A40" s="1" t="s">
-        <v>13</v>
+        <v>109</v>
       </c>
       <c r="B40">
         <v>6</v>
       </c>
       <c r="C40">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="41" spans="1:3">
       <c r="A41" s="1" t="s">
-        <v>26</v>
+        <v>120</v>
       </c>
       <c r="B41">
         <v>6</v>
       </c>
       <c r="C41">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="42" spans="1:3">

</xml_diff>